<commit_message>
Deploying to gh-pages from @ codeforIATI/codelists@6498964892ddc7d3455b1156239b0d1dd3dc3550 🚀
</commit_message>
<xml_diff>
--- a/api/1/clv1/codelist/AidType-category.xlsx
+++ b/api/1/clv1/codelist/AidType-category.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>code</t>
   </si>
@@ -101,6 +101,12 @@
   </si>
   <si>
     <t>Groups a number of contributions that do not give rise to a cross-border flow.</t>
+  </si>
+  <si>
+    <t>J</t>
+  </si>
+  <si>
+    <t>In-kind donation of goods</t>
   </si>
 </sst>
 </file>
@@ -432,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -561,6 +567,17 @@
         <v>10</v>
       </c>
     </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>